<commit_message>
chore: fix nested folder structure (moved project up one level)
</commit_message>
<xml_diff>
--- a/Template User Story schedule .xlsx
+++ b/Template User Story schedule .xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\road_map\PM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58F209EA-FAFF-4314-AF5D-AB078BF00F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03942090-9298-4EAB-862E-CB9E09EA96D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="495">
   <si>
     <t>#story</t>
   </si>
@@ -1640,9 +1640,6 @@
   </si>
   <si>
     <t>27 Sep 2026</t>
-  </si>
-  <si>
-    <t>4 Oct 2026</t>
   </si>
   <si>
     <t>11 Oct 2026</t>
@@ -2807,10 +2804,10 @@
         <v>479</v>
       </c>
       <c r="M5" s="95">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N5" s="97" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="81" customHeight="1" x14ac:dyDescent="0.3">
@@ -2848,7 +2845,7 @@
         <v>2</v>
       </c>
       <c r="N6" s="97" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="81" customHeight="1" x14ac:dyDescent="0.3">
@@ -2886,7 +2883,7 @@
         <v>3</v>
       </c>
       <c r="N7" s="97" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2924,7 +2921,7 @@
         <v>3</v>
       </c>
       <c r="N8" s="97" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
@@ -2962,7 +2959,7 @@
         <v>4</v>
       </c>
       <c r="N9" s="97" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2998,7 +2995,7 @@
         <v>4</v>
       </c>
       <c r="N10" s="97" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -3014,12 +3011,12 @@
       <c r="D11" s="97">
         <v>6</v>
       </c>
-      <c r="E11" s="95" t="s">
-        <v>52</v>
-      </c>
+      <c r="E11" s="95"/>
       <c r="F11" s="95"/>
       <c r="G11" s="95"/>
-      <c r="H11" s="95"/>
+      <c r="H11" s="95" t="s">
+        <v>52</v>
+      </c>
       <c r="I11" s="97" t="s">
         <v>95</v>
       </c>
@@ -3036,7 +3033,7 @@
         <v>5</v>
       </c>
       <c r="N11" s="97" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="67.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -3074,7 +3071,7 @@
         <v>5</v>
       </c>
       <c r="N12" s="97" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="13" spans="1:26" s="98" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
@@ -3112,7 +3109,7 @@
         <v>6</v>
       </c>
       <c r="N13" s="97" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="14" spans="1:26" s="98" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
@@ -3148,7 +3145,7 @@
         <v>6</v>
       </c>
       <c r="N14" s="97" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="15" spans="1:26" s="98" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
@@ -3184,7 +3181,7 @@
         <v>7</v>
       </c>
       <c r="N15" s="97" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="16" spans="1:26" s="98" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
@@ -3220,7 +3217,7 @@
         <v>7</v>
       </c>
       <c r="N16" s="97" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="17" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>